<commit_message>
[Docs] Regenerate VVenC image benchmark charts and table artifacts
</commit_message>
<xml_diff>
--- a/docs/image_benchmark/standard_grayscale/results.xlsx
+++ b/docs/image_benchmark/standard_grayscale/results.xlsx
@@ -588,7 +588,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -598,27 +598,27 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>99281</t>
+          <t>24307</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>3.960636979885376</t>
+          <t>16.17706833422471</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>3.029815673828125</t>
+          <t>0.741790771484375</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>794.248</t>
+          <t>194.456</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>44.189</t>
+          <t>30.4025</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -633,47 +633,47 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>0.995395</t>
+          <t>0.920926</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>49.387</t>
+          <t>35.969</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>96.179678</t>
+          <t>82.739378</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>0.9998454872457103</t>
+          <t>0.9749449175774701</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>0.9969890057772077</t>
+          <t>0.9261632321048087</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>0.9970233851450322</t>
+          <t>0.9274677722744444</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>41.71080163307231</t>
+          <t>28.405409891304714</t>
         </is>
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>43.172571043658195</t>
+          <t>30.35583098745143</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>0.9998303391160142</t>
+          <t>0.974942911631342</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -705,27 +705,27 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>100309</t>
+          <t>24865</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3.920047054601282</t>
+          <t>15.814035793283733</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>3.061187744140625</t>
+          <t>0.758819580078125</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>802.472</t>
+          <t>198.92</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>42.9871</t>
+          <t>29.9047</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -740,54 +740,54 @@
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>0.99393</t>
+          <t>0.915743</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>48.2422</t>
+          <t>35.505</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>96.020386</t>
+          <t>82.374471</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>0.9998363826872788</t>
+          <t>0.9741561537589766</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>0.9959524147239301</t>
+          <t>0.9179577564316944</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>0.9957296972300526</t>
+          <t>0.9163540693043608</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>40.61205709750723</t>
+          <t>27.959221680354382</t>
         </is>
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>42.20944602195593</t>
+          <t>29.867066777733093</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
         <is>
-          <t>0.9998213676485473</t>
+          <t>0.9741542315891518</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>baboon</t>
+          <t>barbara</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -812,27 +812,27 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>71110</t>
+          <t>26515</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>5.529686401350021</t>
+          <t>14.829945313973223</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2.17010498046875</t>
+          <t>0.809173583984375</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>568.88</t>
+          <t>212.12</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>39.2308</t>
+          <t>40.8984</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -847,54 +847,54 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>0.985511</t>
+          <t>0.982372</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>44.5858</t>
+          <t>45.2084</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>94.452705</t>
+          <t>94.435785</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>0.9995319317486188</t>
+          <t>0.9958536873980623</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>0.9898433754795488</t>
+          <t>0.9886703178894095</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>0.9903286633611594</t>
+          <t>0.9918790170666627</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>36.928613482833676</t>
+          <t>38.3264037018021</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>38.871587260579695</t>
+          <t>40.427519668354776</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
         <is>
-          <t>0.9995166222520028</t>
+          <t>0.9958510238168895</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>baboon</t>
+          <t>barbara</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -919,27 +919,27 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>71033</t>
+          <t>26549</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5.5356805991581375</t>
+          <t>14.810953331575577</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2.167755126953125</t>
+          <t>0.810211181640625</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>568.264</t>
+          <t>212.392</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>38.1079</t>
+          <t>40.1341</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -954,47 +954,47 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>0.981436</t>
+          <t>0.980943</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>43.4794</t>
+          <t>44.5584</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>94.417717</t>
+          <t>94.192038</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>0.9994924639844595</t>
+          <t>0.9955608791659207</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>0.986587848098918</t>
+          <t>0.9864541664554837</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>0.986464070865953</t>
+          <t>0.9897225580674069</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>35.858750129772716</t>
+          <t>37.651536313103946</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>37.83702690076686</t>
+          <t>39.74162027074303</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
         <is>
-          <t>0.9994773823799372</t>
+          <t>0.9955582290288536</t>
         </is>
       </c>
     </row>
@@ -1076,7 +1076,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>0.9985418799334178</t>
+          <t>0.9899656408524158</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr">
@@ -1096,12 +1096,12 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>34.39640530895425</t>
+          <t>34.396405308954414</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
         <is>
-          <t>0.9985266538123332</t>
+          <t>0.9899635422645966</t>
         </is>
       </c>
     </row>
@@ -1183,7 +1183,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>0.9984591687067047</t>
+          <t>0.9893812860893489</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr">
@@ -1203,19 +1203,19 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>33.60998689908907</t>
+          <t>33.60998689908918</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
         <is>
-          <t>0.9984438386527689</t>
+          <t>0.9893791659475172</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>baboon</t>
+          <t>barbara</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1240,27 +1240,27 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>24307</t>
+          <t>43875</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>16.17706833422471</t>
+          <t>8.962188034188035</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>0.741790771484375</t>
+          <t>1.338958740234375</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>194.456</t>
+          <t>351.0</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>30.4025</t>
+          <t>44.288</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1275,54 +1275,54 @@
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>0.920926</t>
+          <t>0.990046</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>35.969</t>
+          <t>48.2601</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>82.739378</t>
+          <t>96.067722</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>0.9957819343754036</t>
+          <t>0.9981420035597331</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>0.9261632321048087</t>
+          <t>0.9949497235787337</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>0.9274677722744443</t>
+          <t>0.9964722427201306</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>28.405409891304714</t>
+          <t>41.48957151369512</t>
         </is>
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>30.35583098745149</t>
+          <t>43.31995292519396</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>0.9957671374002891</t>
+          <t>0.9981393193390993</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>baboon</t>
+          <t>barbara</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1347,27 +1347,27 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>24865</t>
+          <t>44537</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>15.814035793283733</t>
+          <t>8.82897366234816</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0.758819580078125</t>
+          <t>1.359161376953125</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>198.92</t>
+          <t>356.296</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>29.9047</t>
+          <t>43.3844</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1382,54 +1382,54 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>0.915743</t>
+          <t>0.988234</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>35.505</t>
+          <t>47.4483</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>82.374471</t>
+          <t>95.935061</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>0.9956173912543701</t>
+          <t>0.9978961269449509</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>0.9179577564316944</t>
+          <t>0.993622457182366</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>0.9163540693043609</t>
+          <t>0.9953464278143517</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>27.959221680354382</t>
+          <t>40.66789649500578</t>
         </is>
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>29.86706677773313</t>
+          <t>42.602106474295525</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
         <is>
-          <t>0.9956032460368696</t>
+          <t>0.9978934927407286</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>barbara</t>
+          <t>baboon</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>27</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1454,27 +1454,27 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>43875</t>
+          <t>71110</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>8.962188034188035</t>
+          <t>5.529686401350021</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>1.338958740234375</t>
+          <t>2.17010498046875</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>351.0</t>
+          <t>568.88</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>44.288</t>
+          <t>39.2308</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1489,54 +1489,54 @@
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>0.990046</t>
+          <t>0.985511</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>48.2601</t>
+          <t>44.5858</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>96.067722</t>
+          <t>94.452705</t>
         </is>
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>0.999882362932024</t>
+          <t>0.9967262860152624</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>0.9949497235787337</t>
+          <t>0.9898433754795488</t>
         </is>
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>0.9964722427201307</t>
+          <t>0.9903286633611594</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>41.48957151369512</t>
+          <t>36.928613482833676</t>
         </is>
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>43.31995292519392</t>
+          <t>38.8715872605799</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
         <is>
-          <t>0.9998638116471802</t>
+          <t>0.9967241505609791</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>barbara</t>
+          <t>baboon</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1551,7 +1551,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>27</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1561,27 +1561,27 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>44537</t>
+          <t>71033</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>8.82897366234816</t>
+          <t>5.5356805991581375</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>1.359161376953125</t>
+          <t>2.167755126953125</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>356.296</t>
+          <t>568.264</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>43.3844</t>
+          <t>38.1079</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1596,54 +1596,54 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>0.988234</t>
+          <t>0.981436</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>47.4483</t>
+          <t>43.4794</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>95.935061</t>
+          <t>94.417717</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>0.9998706815792555</t>
+          <t>0.9962364146999818</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>0.993622457182366</t>
+          <t>0.986587848098918</t>
         </is>
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>0.9953464278143517</t>
+          <t>0.9864640708659529</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>40.66789649500578</t>
+          <t>35.858750129772716</t>
         </is>
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>42.602106474295425</t>
+          <t>37.83702690076706</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
         <is>
-          <t>0.9998524372407424</t>
+          <t>0.9962342990442296</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>barbara</t>
+          <t>baboon</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1658,7 +1658,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1668,27 +1668,27 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>26515</t>
+          <t>99281</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>14.829945313973223</t>
+          <t>3.960636979885376</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>0.809173583984375</t>
+          <t>3.029815673828125</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>212.12</t>
+          <t>794.248</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>40.8984</t>
+          <t>44.189</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -1703,54 +1703,54 @@
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>0.982372</t>
+          <t>0.995395</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>45.2084</t>
+          <t>49.387</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>94.435785</t>
+          <t>96.179678</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>0.9997108577447585</t>
+          <t>0.9989910345685677</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>0.9886703178894095</t>
+          <t>0.9969890057772077</t>
         </is>
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>0.9918790170666627</t>
+          <t>0.9970233851450322</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>38.3264037018021</t>
+          <t>41.71080163307231</t>
         </is>
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>40.4275196683545</t>
+          <t>43.17257104365818</t>
         </is>
       </c>
       <c r="U12" t="inlineStr">
         <is>
-          <t>0.9996923804925277</t>
+          <t>0.9989889104794761</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>barbara</t>
+          <t>baboon</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1765,7 +1765,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1775,27 +1775,27 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>26549</t>
+          <t>100309</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>14.810953331575577</t>
+          <t>3.920047054601282</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0.810211181640625</t>
+          <t>3.061187744140625</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>212.392</t>
+          <t>802.472</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>40.1341</t>
+          <t>42.9871</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1810,47 +1810,47 @@
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>0.980943</t>
+          <t>0.99393</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>44.5584</t>
+          <t>48.2422</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>94.192038</t>
+          <t>96.020386</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>0.9996805415125324</t>
+          <t>0.99888648958426</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>0.9864541664554837</t>
+          <t>0.9959524147239301</t>
         </is>
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>0.9897225580674069</t>
+          <t>0.9957296972300526</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>37.651536313103946</t>
+          <t>40.61205709750723</t>
         </is>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>39.74162027074264</t>
+          <t>42.20944602195593</t>
         </is>
       </c>
       <c r="U13" t="inlineStr">
         <is>
-          <t>0.9996621594413821</t>
+          <t>0.9988843872943031</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>0.999305638071036</t>
+          <t>0.9915894911218223</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr">
@@ -1942,7 +1942,7 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>0.9841815499986263</t>
+          <t>0.9841815499986262</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1952,12 +1952,12 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>37.69242937667337</t>
+          <t>37.69242937667371</t>
         </is>
       </c>
       <c r="U14" t="inlineStr">
         <is>
-          <t>0.9992874112896147</t>
+          <t>0.9915868771093376</t>
         </is>
       </c>
     </row>
@@ -2039,7 +2039,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>0.9992335233493114</t>
+          <t>0.9910253970370457</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>0.9798354541365644</t>
+          <t>0.9798354541365643</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -2059,12 +2059,12 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>36.919352047535234</t>
+          <t>36.919352047535504</t>
         </is>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>0.9992155106175643</t>
+          <t>0.991022802459919</t>
         </is>
       </c>
     </row>
@@ -2146,7 +2146,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>0.9983139605594052</t>
+          <t>0.9834859595463773</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr">
@@ -2166,12 +2166,12 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>34.6471189390268</t>
+          <t>34.6471189390269</t>
         </is>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>0.998295867837505</t>
+          <t>0.9834833823242685</t>
         </is>
       </c>
     </row>
@@ -2253,7 +2253,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>0.9981721945283275</t>
+          <t>0.9826259849946682</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr">
@@ -2263,7 +2263,7 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>0.9588389118018562</t>
+          <t>0.9588389118018563</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2273,12 +2273,12 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>33.79736103715188</t>
+          <t>33.79736103715193</t>
         </is>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>0.9981533981802402</t>
+          <t>0.9826233143728139</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -2310,27 +2310,27 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>57189</t>
+          <t>7598</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>6.875727849761318</t>
+          <t>51.75256646485917</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>1.745269775390625</t>
+          <t>0.23187255859375</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>457.512</t>
+          <t>60.784</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>44.1648</t>
+          <t>33.2317</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -2345,47 +2345,47 @@
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>0.990488</t>
+          <t>0.912516</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>47.7707</t>
+          <t>37.0981</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>96.001199</t>
+          <t>83.880815</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>0.9998966482243016</t>
+          <t>0.9711962946677782</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>0.9915970170076085</t>
+          <t>0.8870013163099878</t>
         </is>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>0.994628104222054</t>
+          <t>0.9315842103903013</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>41.13126227640234</t>
+          <t>30.541523588385985</t>
         </is>
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>43.241587373791916</t>
+          <t>33.15196285158254</t>
         </is>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>0.9998783423507426</t>
+          <t>0.9711936262705679</t>
         </is>
       </c>
     </row>
@@ -2407,7 +2407,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2417,27 +2417,27 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>55661</t>
+          <t>7983</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>7.064479617685633</t>
+          <t>49.256670424652384</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>1.698638916015625</t>
+          <t>0.243621826171875</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>445.288</t>
+          <t>63.864</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>42.9815</t>
+          <t>33.0238</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -2452,47 +2452,47 @@
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>0.987752</t>
+          <t>0.909441</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>46.6146</t>
+          <t>36.9183</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>96.002478</t>
+          <t>83.439058</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0.9998834427103005</t>
+          <t>0.9704959817752608</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>0.9886817387048942</t>
+          <t>0.8814756565909498</t>
         </is>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>0.9924110806587537</t>
+          <t>0.9277507996115979</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>40.012662676550725</t>
+          <t>30.339203055064385</t>
         </is>
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>42.25338325761052</t>
+          <t>32.9450019220455</t>
         </is>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>0.9998650305404557</t>
+          <t>0.970493202410675</t>
         </is>
       </c>
     </row>
@@ -2514,7 +2514,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>32</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2524,27 +2524,27 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>32124</t>
+          <t>15921</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>12.240567799775869</t>
+          <t>24.697946108912756</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>0.9803466796875</t>
+          <t>0.485870361328125</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>256.992</t>
+          <t>127.368</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>39.6423</t>
+          <t>36.0617</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -2559,47 +2559,47 @@
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>0.975844</t>
+          <t>0.950177</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>43.3553</t>
+          <t>39.862</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>94.289785</t>
+          <t>91.171464</t>
         </is>
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>0.999707323709047</t>
+          <t>0.9870041259803232</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>0.9745570201355785</t>
+          <t>0.9394801035775086</t>
         </is>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>0.9837130101453431</t>
+          <t>0.9617739349356649</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>36.78946198368887</t>
+          <t>33.29506179708248</t>
         </is>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>39.31196387938022</t>
+          <t>35.907363690092104</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>0.9996896103257263</t>
+          <t>0.9870013232158469</t>
         </is>
       </c>
     </row>
@@ -2621,7 +2621,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>32</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -2631,27 +2631,27 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>30924</t>
+          <t>15796</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>12.715560729530461</t>
+          <t>24.893390731830845</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0.9437255859375</t>
+          <t>0.4820556640625</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>247.392</t>
+          <t>126.368</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>38.9141</t>
+          <t>35.6531</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -2666,47 +2666,47 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>0.972209</t>
+          <t>0.946409</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>42.6652</t>
+          <t>39.4765</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>94.133335</t>
+          <t>90.834361</t>
         </is>
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>0.9996767978975839</t>
+          <t>0.9862559480242484</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>0.9691297732545303</t>
+          <t>0.933169966625367</t>
         </is>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>0.9796981522398333</t>
+          <t>0.9573030189695116</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>36.088655490929696</t>
+          <t>32.9038956464188</t>
         </is>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>38.62572394183235</t>
+          <t>35.5131187449106</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>0.9996587778303069</t>
+          <t>0.986253092163803</t>
         </is>
       </c>
     </row>
@@ -2728,7 +2728,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>27</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -2738,27 +2738,27 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>15921</t>
+          <t>32124</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>24.697946108912756</t>
+          <t>12.240567799775869</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>0.485870361328125</t>
+          <t>0.9803466796875</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>127.368</t>
+          <t>256.992</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>36.0617</t>
+          <t>39.6423</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -2773,47 +2773,47 @@
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>0.950177</t>
+          <t>0.975844</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>39.862</t>
+          <t>43.3553</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>91.171464</t>
+          <t>94.289785</t>
         </is>
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>0.999211482334083</t>
+          <t>0.99486259664232</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr">
         <is>
-          <t>0.9394801035775086</t>
+          <t>0.9745570201355785</t>
         </is>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>0.9617739349356648</t>
+          <t>0.9837130101453431</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>33.29506179708248</t>
+          <t>36.78946198368887</t>
         </is>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>35.90736369009191</t>
+          <t>39.311963879380535</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>0.9991934553809273</t>
+          <t>0.9948598117390849</t>
         </is>
       </c>
     </row>
@@ -2835,7 +2835,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>27</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -2845,27 +2845,27 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>15796</t>
+          <t>30924</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>24.893390731830845</t>
+          <t>12.715560729530461</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.4820556640625</t>
+          <t>0.9437255859375</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>126.368</t>
+          <t>247.392</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>35.6531</t>
+          <t>38.9141</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -2880,47 +2880,47 @@
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>0.946409</t>
+          <t>0.972209</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>39.4765</t>
+          <t>42.6652</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>90.834361</t>
+          <t>94.133335</t>
         </is>
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>0.9991570621770278</t>
+          <t>0.9942739913000552</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr">
         <is>
-          <t>0.933169966625367</t>
+          <t>0.9691297732545303</t>
         </is>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>0.9573030189695116</t>
+          <t>0.9796981522398333</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>32.9038956464188</t>
+          <t>36.088655490929696</t>
         </is>
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>35.5131187449105</t>
+          <t>38.625723941832675</t>
         </is>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>0.9991390140354616</t>
+          <t>0.9942711281897868</t>
         </is>
       </c>
     </row>
@@ -2942,7 +2942,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -2952,27 +2952,27 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>7598</t>
+          <t>57189</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>51.75256646485917</t>
+          <t>6.875727849761318</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>0.23187255859375</t>
+          <t>1.745269775390625</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>60.784</t>
+          <t>457.512</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>33.2317</t>
+          <t>44.1648</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -2987,47 +2987,47 @@
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>0.912516</t>
+          <t>0.990488</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>37.0981</t>
+          <t>47.7707</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>83.880815</t>
+          <t>96.001199</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>0.998078527865899</t>
+          <t>0.9981703394433422</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr">
         <is>
-          <t>0.8870013163099878</t>
+          <t>0.9915970170076085</t>
         </is>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>0.9315842103903013</t>
+          <t>0.994628104222054</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>30.541523588385985</t>
+          <t>41.13126227640233</t>
         </is>
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>33.151962851582425</t>
+          <t>43.24158737379186</t>
         </is>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>0.9980608127326777</t>
+          <t>0.9981674231711394</t>
         </is>
       </c>
     </row>
@@ -3049,7 +3049,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3059,27 +3059,27 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>7983</t>
+          <t>55661</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>49.256670424652384</t>
+          <t>7.064479617685633</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>0.243621826171875</t>
+          <t>1.698638916015625</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>63.864</t>
+          <t>445.288</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>33.0238</t>
+          <t>42.9815</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -3094,47 +3094,47 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>0.909441</t>
+          <t>0.987752</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>36.9183</t>
+          <t>46.6146</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>83.439058</t>
+          <t>96.002478</t>
         </is>
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>0.9980132314280453</t>
+          <t>0.9978758116798984</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr">
         <is>
-          <t>0.8814756565909498</t>
+          <t>0.9886817387048942</t>
         </is>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>0.9277507996115979</t>
+          <t>0.9924110806587537</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>30.339203055064385</t>
+          <t>40.012662676550725</t>
         </is>
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>32.9450019220454</t>
+          <t>42.25338325761058</t>
         </is>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>0.9979951683782655</t>
+          <t>0.9978728862882402</t>
         </is>
       </c>
     </row>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -3166,27 +3166,27 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>37586</t>
+          <t>4953</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>10.461767679455116</t>
+          <t>79.38946093276802</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1.14703369140625</t>
+          <t>0.151153564453125</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>300.688</t>
+          <t>39.624</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>44.0718</t>
+          <t>35.7766</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -3201,47 +3201,47 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>0.985132</t>
+          <t>0.942794</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>47.9026</t>
+          <t>39.7353</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>96.471093</t>
+          <t>85.433024</t>
         </is>
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>0.9998880835714763</t>
+          <t>0.9813929449227131</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr">
         <is>
-          <t>0.9890625522119305</t>
+          <t>0.9217611297051176</t>
         </is>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>0.994081613584004</t>
+          <t>0.9561288832899648</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>40.984759741058376</t>
+          <t>33.17530826927151</t>
         </is>
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>43.13260577098406</t>
+          <t>35.61607569746289</t>
         </is>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>0.9998723361840179</t>
+          <t>0.9813906227371181</t>
         </is>
       </c>
     </row>
@@ -3263,7 +3263,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -3273,27 +3273,27 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>34819</t>
+          <t>5545</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>11.29314454751716</t>
+          <t>70.9136158701533</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>1.062591552734375</t>
+          <t>0.169219970703125</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>278.552</t>
+          <t>44.36</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>43.0446</t>
+          <t>35.6456</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -3308,47 +3308,47 @@
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>0.981563</t>
+          <t>0.942468</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>46.8793</t>
+          <t>39.6029</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>96.364874</t>
+          <t>85.781859</t>
         </is>
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>0.9998735218198902</t>
+          <t>0.9814259085058971</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr">
         <is>
-          <t>0.9853852253511047</t>
+          <t>0.9196384090847023</t>
         </is>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>0.9919344264301269</t>
+          <t>0.9543529458723345</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>40.01009077890333</t>
+          <t>33.063800344143296</t>
         </is>
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>42.27027579071592</t>
+          <t>35.492114111284565</t>
         </is>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>0.9998575404830987</t>
+          <t>0.9814236119220435</t>
         </is>
       </c>
     </row>
@@ -3430,7 +3430,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>0.9997139392948775</t>
+          <t>0.9935580308455694</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr">
@@ -3450,12 +3450,12 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>39.98740324444873</t>
+          <t>39.98740324444903</t>
         </is>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>0.9996982274845959</t>
+          <t>0.9935557716851632</t>
         </is>
       </c>
     </row>
@@ -3537,7 +3537,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>0.9996989861870667</t>
+          <t>0.9933031043760897</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr">
@@ -3547,7 +3547,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>0.9827177635812879</t>
+          <t>0.9827177635812878</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -3557,12 +3557,12 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>39.68580824182159</t>
+          <t>39.68580824182192</t>
         </is>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>0.9996831106721334</t>
+          <t>0.9933008209830758</t>
         </is>
       </c>
     </row>
@@ -3644,7 +3644,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>0.9993940150008302</t>
+          <t>0.9889166422302181</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr">
@@ -3664,12 +3664,12 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>37.81933148632162</t>
+          <t>37.819331486321865</t>
         </is>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>0.9993781556020621</t>
+          <t>0.9889143612392143</t>
         </is>
       </c>
     </row>
@@ -3751,7 +3751,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>0.999371193526864</t>
+          <t>0.988663819195445</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr">
@@ -3771,12 +3771,12 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>37.59804353102068</t>
+          <t>37.59804353102089</t>
         </is>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>0.9993553751221743</t>
+          <t>0.9886615533312986</t>
         </is>
       </c>
     </row>
@@ -3798,7 +3798,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -3808,27 +3808,27 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>4953</t>
+          <t>37586</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>79.38946093276802</t>
+          <t>10.461767679455116</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>0.151153564453125</t>
+          <t>1.14703369140625</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>39.624</t>
+          <t>300.688</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>35.7766</t>
+          <t>44.0718</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -3843,47 +3843,47 @@
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>0.942794</t>
+          <t>0.985132</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>39.7353</t>
+          <t>47.9026</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>85.433024</t>
+          <t>96.471093</t>
         </is>
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>0.9987073058140373</t>
+          <t>0.9973299995622926</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr">
         <is>
-          <t>0.9217611297051176</t>
+          <t>0.9890625522119305</t>
         </is>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>0.9561288832899649</t>
+          <t>0.9940816135840042</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>33.17530826927151</t>
+          <t>40.984759741058376</t>
         </is>
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>35.616075697462804</t>
+          <t>43.13260577098422</t>
         </is>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>0.9986910263989888</t>
+          <t>0.9973277177087271</t>
         </is>
       </c>
     </row>
@@ -3905,7 +3905,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3915,27 +3915,27 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>5545</t>
+          <t>34819</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>70.9136158701533</t>
+          <t>11.29314454751716</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>0.169219970703125</t>
+          <t>1.062591552734375</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>44.36</t>
+          <t>278.552</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>35.6456</t>
+          <t>43.0446</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -3950,47 +3950,47 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>0.942468</t>
+          <t>0.981563</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>39.6029</t>
+          <t>46.8793</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>85.781859</t>
+          <t>96.364874</t>
         </is>
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>0.9986812223393419</t>
+          <t>0.9968609329744322</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr">
         <is>
-          <t>0.9196384090847023</t>
+          <t>0.9853852253511047</t>
         </is>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>0.9543529458723345</t>
+          <t>0.9919344264301267</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>33.063800344143296</t>
+          <t>40.01009077890333</t>
         </is>
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>35.49211411128456</t>
+          <t>42.27027579071609</t>
         </is>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>0.9986651731673498</t>
+          <t>0.9968586104425636</t>
         </is>
       </c>
     </row>
@@ -4012,7 +4012,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -4022,27 +4022,27 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>49494</t>
+          <t>4649</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>7.944720572190569</t>
+          <t>84.58077005807701</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>1.51043701171875</t>
+          <t>0.141876220703125</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>395.952</t>
+          <t>37.192</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>44.2514</t>
+          <t>35.0229</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -4057,47 +4057,47 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>0.986826</t>
+          <t>0.924583</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>47.9395</t>
+          <t>38.9528</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>96.62577</t>
+          <t>88.019663</t>
         </is>
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>0.9999121754696663</t>
+          <t>0.9795718494217857</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr">
         <is>
-          <t>0.9897997259561444</t>
+          <t>0.9094007881156904</t>
         </is>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>0.9945897598551133</t>
+          <t>0.9486284939176921</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>41.19168128308978</t>
+          <t>32.41224110838026</t>
         </is>
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>43.2698081029622</t>
+          <t>34.87122206706833</t>
         </is>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>0.9998955924169183</t>
+          <t>0.9795692199652756</t>
         </is>
       </c>
     </row>
@@ -4119,7 +4119,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>37</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -4129,27 +4129,27 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>48901</t>
+          <t>5299</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>8.041062554957977</t>
+          <t>74.20569918852614</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>1.492340087890625</t>
+          <t>0.161712646484375</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>391.208</t>
+          <t>42.392</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>42.8141</t>
+          <t>34.9885</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -4164,47 +4164,47 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>0.98118</t>
+          <t>0.924569</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>46.5621</t>
+          <t>38.924</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>96.349755</t>
+          <t>87.297655</t>
         </is>
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>0.9999020605405602</t>
+          <t>0.9796106118934751</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr">
         <is>
-          <t>0.985947559852231</t>
+          <t>0.9092963512981739</t>
         </is>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>0.9916754647863252</t>
+          <t>0.9483179624110316</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>39.83890407811757</t>
+          <t>32.3992407347341</t>
         </is>
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>42.097542115987416</t>
+          <t>34.84490071959452</t>
         </is>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>0.9998855827843677</t>
+          <t>0.9796080224790273</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>32</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -4236,27 +4236,27 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>21724</t>
+          <t>8307</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>18.100533971644264</t>
+          <t>47.335500180570605</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>0.6629638671875</t>
+          <t>0.253509521484375</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>173.792</t>
+          <t>66.456</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>39.4552</t>
+          <t>36.6239</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -4271,47 +4271,47 @@
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>0.962514</t>
+          <t>0.937291</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>43.2197</t>
+          <t>40.4652</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>95.415551</t>
+          <t>92.826336</t>
         </is>
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>0.9997455065179982</t>
+          <t>0.9861858075639875</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr">
         <is>
-          <t>0.9642445305678892</t>
+          <t>0.930753194142375</t>
         </is>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>0.9815310529452246</t>
+          <t>0.9609148756535569</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>36.589326661792654</t>
+          <t>33.8807612984594</t>
         </is>
       </c>
       <c r="T36" t="inlineStr">
         <is>
-          <t>39.10378970978052</t>
+          <t>36.427385553292496</t>
         </is>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>0.9997288979558338</t>
+          <t>0.986183286120078</t>
         </is>
       </c>
     </row>
@@ -4333,7 +4333,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>27</t>
+          <t>32</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -4343,27 +4343,27 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>18602</t>
+          <t>8772</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>21.13837221804107</t>
+          <t>44.82626538987688</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>0.56768798828125</t>
+          <t>0.2677001953125</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>148.816</t>
+          <t>70.176</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>38.4232</t>
+          <t>36.5232</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -4378,47 +4378,47 @@
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>0.952621</t>
+          <t>0.936841</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>42.2167</t>
+          <t>40.3787</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>95.501385</t>
+          <t>92.91153</t>
         </is>
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>0.9997170025627538</t>
+          <t>0.9860406502714524</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr">
         <is>
-          <t>0.9550276042667241</t>
+          <t>0.9295786046765885</t>
         </is>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>0.9735844651399831</t>
+          <t>0.9598549611418101</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>35.57913841149112</t>
+          <t>33.802683014237346</t>
         </is>
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>38.14382446845897</t>
+          <t>36.33988993809178</t>
         </is>
       </c>
       <c r="U37" t="inlineStr">
         <is>
-          <t>0.9997003751948131</t>
+          <t>0.9860381960367214</t>
         </is>
       </c>
     </row>
@@ -4440,7 +4440,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>27</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -4450,27 +4450,27 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>8307</t>
+          <t>21724</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>47.335500180570605</t>
+          <t>18.100533971644264</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>0.253509521484375</t>
+          <t>0.6629638671875</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>66.456</t>
+          <t>173.792</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>36.6239</t>
+          <t>39.4552</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -4485,47 +4485,47 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>0.937291</t>
+          <t>0.962514</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>40.4652</t>
+          <t>43.2197</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>92.826336</t>
+          <t>95.415551</t>
         </is>
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>0.9994308037239357</t>
+          <t>0.9927267848144179</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr">
         <is>
-          <t>0.930753194142375</t>
+          <t>0.9642445305678892</t>
         </is>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>0.960914875653557</t>
+          <t>0.9815310529452246</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>33.8807612984594</t>
+          <t>36.589326661792654</t>
         </is>
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>36.42738555329221</t>
+          <t>39.10378970978075</t>
         </is>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>0.9994138040623417</t>
+          <t>0.9927243058636522</t>
         </is>
       </c>
     </row>
@@ -4547,7 +4547,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>27</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -4557,27 +4557,27 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>8772</t>
+          <t>18602</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>44.82626538987688</t>
+          <t>21.13837221804107</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>0.2677001953125</t>
+          <t>0.56768798828125</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>70.176</t>
+          <t>148.816</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>36.5232</t>
+          <t>38.4232</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -4592,47 +4592,47 @@
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>0.936841</t>
+          <t>0.952621</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>40.3787</t>
+          <t>42.2167</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>92.91153</t>
+          <t>95.501385</t>
         </is>
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>0.9994221592843042</t>
+          <t>0.9916822727242347</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr">
         <is>
-          <t>0.9295786046765885</t>
+          <t>0.9550276042667241</t>
         </is>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>0.95985496114181</t>
+          <t>0.9735844651399831</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>33.802683014237346</t>
+          <t>35.57913841149112</t>
         </is>
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>36.33988993809157</t>
+          <t>38.143824468459314</t>
         </is>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>0.999405557595226</t>
+          <t>0.9916797902179987</t>
         </is>
       </c>
     </row>
@@ -4654,7 +4654,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -4664,27 +4664,27 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>4649</t>
+          <t>49494</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>84.58077005807701</t>
+          <t>7.944720572190569</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>0.141876220703125</t>
+          <t>1.51043701171875</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>37.192</t>
+          <t>395.952</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>35.0229</t>
+          <t>44.2514</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -4699,47 +4699,47 @@
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>0.924583</t>
+          <t>0.986826</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>38.9528</t>
+          <t>47.9395</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>88.019663</t>
+          <t>96.62577</t>
         </is>
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>0.9989042183376833</t>
+          <t>0.9976386549286708</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr">
         <is>
-          <t>0.9094007881156904</t>
+          <t>0.9897997259561444</t>
         </is>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>0.9486284939176921</t>
+          <t>0.9945897598551134</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>32.41224110838026</t>
+          <t>41.19168128308978</t>
         </is>
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>34.87122206706824</t>
+          <t>43.26980810296212</t>
         </is>
       </c>
       <c r="U40" t="inlineStr">
         <is>
-          <t>0.9988863229583659</t>
+          <t>0.997636168066515</t>
         </is>
       </c>
     </row>
@@ -4761,7 +4761,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>22</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -4771,27 +4771,27 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>5299</t>
+          <t>48901</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>74.20569918852614</t>
+          <t>8.041062554957977</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>0.161712646484375</t>
+          <t>1.492340087890625</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>42.392</t>
+          <t>391.208</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>34.9885</t>
+          <t>42.8141</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -4806,47 +4806,47 @@
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>0.924569</t>
+          <t>0.98118</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>38.924</t>
+          <t>46.5621</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>87.297655</t>
+          <t>96.349755</t>
         </is>
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>0.9989067614410446</t>
+          <t>0.9971556084084445</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr">
         <is>
-          <t>0.9092963512981739</t>
+          <t>0.985947559852231</t>
         </is>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>0.9483179624110316</t>
+          <t>0.9916754647863253</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>32.3992407347341</t>
+          <t>39.83890407811757</t>
         </is>
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>34.84490071959441</t>
+          <t>42.09754211598754</t>
         </is>
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>0.9988892210350441</t>
+          <t>0.9971531483920776</t>
         </is>
       </c>
     </row>
@@ -4999,7 +4999,7 @@
         <v>-0.1592919999999935</v>
       </c>
       <c r="K2" t="n">
-        <v>-9.104558431505261e-06</v>
+        <v>-0.0001045449843077861</v>
       </c>
       <c r="L2" t="n">
         <v>-0.00103659105327758</v>
@@ -5011,10 +5011,10 @@
         <v>-1.098744535565075</v>
       </c>
       <c r="O2" t="n">
-        <v>-0.9631250217022682</v>
+        <v>-0.963125021702254</v>
       </c>
       <c r="P2" t="n">
-        <v>-8.971467466811767e-06</v>
+        <v>-0.0001045231851730666</v>
       </c>
     </row>
     <row r="3">
@@ -5051,22 +5051,22 @@
         <v>-0.03498799999999846</v>
       </c>
       <c r="K3" t="n">
-        <v>-3.946776415930664e-05</v>
+        <v>-0.0004898713152805545</v>
       </c>
       <c r="L3" t="n">
         <v>-0.00325552738063084</v>
       </c>
       <c r="M3" t="n">
-        <v>-0.003864592495206431</v>
+        <v>-0.003864592495206542</v>
       </c>
       <c r="N3" t="n">
         <v>-1.06986335306096</v>
       </c>
       <c r="O3" t="n">
-        <v>-1.034560359812836</v>
+        <v>-1.034560359812843</v>
       </c>
       <c r="P3" t="n">
-        <v>-3.923987206555513e-05</v>
+        <v>-0.0004898515167495177</v>
       </c>
     </row>
     <row r="4">
@@ -5103,7 +5103,7 @@
         <v>0.1401180000000011</v>
       </c>
       <c r="K4" t="n">
-        <v>-8.271122671310582e-05</v>
+        <v>-0.0005843547630668411</v>
       </c>
       <c r="L4" t="n">
         <v>-0.006389905334788226</v>
@@ -5115,10 +5115,10 @@
         <v>-0.7575345657614996</v>
       </c>
       <c r="O4" t="n">
-        <v>-0.7864184098651776</v>
+        <v>-0.7864184098652345</v>
       </c>
       <c r="P4" t="n">
-        <v>-8.281515956432006e-05</v>
+        <v>-0.0005843763170794158</v>
       </c>
     </row>
     <row r="5">
@@ -5155,22 +5155,22 @@
         <v>-0.3649070000000023</v>
       </c>
       <c r="K5" t="n">
-        <v>-0.0001645431210335335</v>
+        <v>-0.0007887638184935764</v>
       </c>
       <c r="L5" t="n">
         <v>-0.008205475673114249</v>
       </c>
       <c r="M5" t="n">
-        <v>-0.01111370297008341</v>
+        <v>-0.01111370297008363</v>
       </c>
       <c r="N5" t="n">
         <v>-0.4461882109503321</v>
       </c>
       <c r="O5" t="n">
-        <v>-0.4887642097183615</v>
+        <v>-0.4887642097183367</v>
       </c>
       <c r="P5" t="n">
-        <v>-0.0001638913634195438</v>
+        <v>-0.0007886800421901263</v>
       </c>
     </row>
     <row r="6">
@@ -5207,22 +5207,22 @@
         <v>-0.1326609999999988</v>
       </c>
       <c r="K6" t="n">
-        <v>-1.168135276852222e-05</v>
+        <v>-0.0002458766147822589</v>
       </c>
       <c r="L6" t="n">
         <v>-0.00132726639636771</v>
       </c>
       <c r="M6" t="n">
-        <v>-0.00112581490577901</v>
+        <v>-0.001125814905778899</v>
       </c>
       <c r="N6" t="n">
         <v>-0.8216750186893407</v>
       </c>
       <c r="O6" t="n">
-        <v>-0.7178464508984916</v>
+        <v>-0.7178464508984348</v>
       </c>
       <c r="P6" t="n">
-        <v>-1.137440643783627e-05</v>
+        <v>-0.0002458265983706909</v>
       </c>
     </row>
     <row r="7">
@@ -5259,7 +5259,7 @@
         <v>-0.243746999999999</v>
       </c>
       <c r="K7" t="n">
-        <v>-3.031623222615742e-05</v>
+        <v>-0.000292808232141617</v>
       </c>
       <c r="L7" t="n">
         <v>-0.002216151433925839</v>
@@ -5271,10 +5271,10 @@
         <v>-0.6748673886981535</v>
       </c>
       <c r="O7" t="n">
-        <v>-0.6858993976118626</v>
+        <v>-0.6858993976117489</v>
       </c>
       <c r="P7" t="n">
-        <v>-3.022105114558471e-05</v>
+        <v>-0.0002927947880358994</v>
       </c>
     </row>
     <row r="8">
@@ -5311,7 +5311,7 @@
         <v>0.02558399999999494</v>
       </c>
       <c r="K8" t="n">
-        <v>-7.211472172463651e-05</v>
+        <v>-0.0005640940847765341</v>
       </c>
       <c r="L8" t="n">
         <v>-0.004226607587413889</v>
@@ -5323,10 +5323,10 @@
         <v>-0.7358560109999317</v>
       </c>
       <c r="O8" t="n">
-        <v>-0.7730773291381325</v>
+        <v>-0.7730773291382036</v>
       </c>
       <c r="P8" t="n">
-        <v>-7.190067205042894e-05</v>
+        <v>-0.0005640746494185445</v>
       </c>
     </row>
     <row r="9">
@@ -5363,22 +5363,22 @@
         <v>-0.3988130000000041</v>
       </c>
       <c r="K9" t="n">
-        <v>-0.0001417660310777391</v>
+        <v>-0.0008599745517090529</v>
       </c>
       <c r="L9" t="n">
         <v>-0.01066348420458685</v>
       </c>
       <c r="M9" t="n">
-        <v>-0.009822788726455811</v>
+        <v>-0.0098227887264557</v>
       </c>
       <c r="N9" t="n">
         <v>-0.8033603069415776</v>
       </c>
       <c r="O9" t="n">
-        <v>-0.8497579018749164</v>
+        <v>-0.8497579018749732</v>
       </c>
       <c r="P9" t="n">
-        <v>-0.0001424696572648321</v>
+        <v>-0.0008600679514545462</v>
       </c>
     </row>
     <row r="10">
@@ -5415,7 +5415,7 @@
         <v>0.001278999999996699</v>
       </c>
       <c r="K10" t="n">
-        <v>-1.320551400108005e-05</v>
+        <v>-0.0002945277634438526</v>
       </c>
       <c r="L10" t="n">
         <v>-0.002915278302714319</v>
@@ -5424,13 +5424,13 @@
         <v>-0.002217023563300335</v>
       </c>
       <c r="N10" t="n">
-        <v>-1.118599599851613</v>
+        <v>-1.118599599851606</v>
       </c>
       <c r="O10" t="n">
-        <v>-0.988204116181393</v>
+        <v>-0.9882041161812793</v>
       </c>
       <c r="P10" t="n">
-        <v>-1.331181028685346e-05</v>
+        <v>-0.0002945368828991546</v>
       </c>
     </row>
     <row r="11">
@@ -5467,7 +5467,7 @@
         <v>-0.1564499999999924</v>
       </c>
       <c r="K11" t="n">
-        <v>-3.052581146312239e-05</v>
+        <v>-0.0005886053422647919</v>
       </c>
       <c r="L11" t="n">
         <v>-0.005427246881048231</v>
@@ -5479,10 +5479,10 @@
         <v>-0.7008064927591704</v>
       </c>
       <c r="O11" t="n">
-        <v>-0.6862399375478745</v>
+        <v>-0.6862399375478603</v>
       </c>
       <c r="P11" t="n">
-        <v>-3.083249541946387e-05</v>
+        <v>-0.0005886835492980858</v>
       </c>
     </row>
     <row r="12">
@@ -5519,22 +5519,22 @@
         <v>-0.337102999999999</v>
       </c>
       <c r="K12" t="n">
-        <v>-5.442015705514613e-05</v>
+        <v>-0.0007481779560747359</v>
       </c>
       <c r="L12" t="n">
         <v>-0.006310136952141554</v>
       </c>
       <c r="M12" t="n">
-        <v>-0.004470915966153122</v>
+        <v>-0.004470915966153233</v>
       </c>
       <c r="N12" t="n">
         <v>-0.391166150663679</v>
       </c>
       <c r="O12" t="n">
-        <v>-0.3942449451814127</v>
+        <v>-0.3942449451815051</v>
       </c>
       <c r="P12" t="n">
-        <v>-5.444134546572776e-05</v>
+        <v>-0.0007482310520439128</v>
       </c>
     </row>
     <row r="13">
@@ -5571,7 +5571,7 @@
         <v>-0.4417569999999955</v>
       </c>
       <c r="K13" t="n">
-        <v>-6.529643785369021e-05</v>
+        <v>-0.0007003128925174851</v>
       </c>
       <c r="L13" t="n">
         <v>-0.005525659719037956</v>
@@ -5583,10 +5583,10 @@
         <v>-0.2023205333216005</v>
       </c>
       <c r="O13" t="n">
-        <v>-0.2069609295370256</v>
+        <v>-0.2069609295370398</v>
       </c>
       <c r="P13" t="n">
-        <v>-6.564435441214211e-05</v>
+        <v>-0.0007004238598928847</v>
       </c>
     </row>
     <row r="14">
@@ -5623,22 +5623,22 @@
         <v>-0.1062189999999958</v>
       </c>
       <c r="K14" t="n">
-        <v>-1.456175158609518e-05</v>
+        <v>-0.0004690665878603895</v>
       </c>
       <c r="L14" t="n">
         <v>-0.00367732686082578</v>
       </c>
       <c r="M14" t="n">
-        <v>-0.002147187153877184</v>
+        <v>-0.002147187153877406</v>
       </c>
       <c r="N14" t="n">
         <v>-0.9746689621550431</v>
       </c>
       <c r="O14" t="n">
-        <v>-0.8623299802681359</v>
+        <v>-0.8623299802681288</v>
       </c>
       <c r="P14" t="n">
-        <v>-1.479570091922344e-05</v>
+        <v>-0.0004691072661634488</v>
       </c>
     </row>
     <row r="15">
@@ -5675,22 +5675,22 @@
         <v>0.005049999999997112</v>
       </c>
       <c r="K15" t="n">
-        <v>-1.495310781085557e-05</v>
+        <v>-0.000254926469479666</v>
       </c>
       <c r="L15" t="n">
         <v>-0.002681713374285799</v>
       </c>
       <c r="M15" t="n">
-        <v>-0.001881232983296233</v>
+        <v>-0.001881232983296344</v>
       </c>
       <c r="N15" t="n">
         <v>-0.3029923199923132</v>
       </c>
       <c r="O15" t="n">
-        <v>-0.3015950026271383</v>
+        <v>-0.3015950026271099</v>
       </c>
       <c r="P15" t="n">
-        <v>-1.511681246246788e-05</v>
+        <v>-0.0002549507020873643</v>
       </c>
     </row>
     <row r="16">
@@ -5727,7 +5727,7 @@
         <v>-0.3444320000000118</v>
       </c>
       <c r="K16" t="n">
-        <v>-2.282147396626133e-05</v>
+        <v>-0.0002528230347731419</v>
       </c>
       <c r="L16" t="n">
         <v>-0.003178027611734913</v>
@@ -5739,10 +5739,10 @@
         <v>-0.2021375561746552</v>
       </c>
       <c r="O16" t="n">
-        <v>-0.2212879553009444</v>
+        <v>-0.2212879553009728</v>
       </c>
       <c r="P16" t="n">
-        <v>-2.278047988779619e-05</v>
+        <v>-0.0002528079079157086</v>
       </c>
     </row>
     <row r="17">
@@ -5779,22 +5779,22 @@
         <v>0.348834999999994</v>
       </c>
       <c r="K17" t="n">
-        <v>-2.608347469545969e-05</v>
+        <v>3.296358318394255e-05</v>
       </c>
       <c r="L17" t="n">
         <v>-0.002122720620415297</v>
       </c>
       <c r="M17" t="n">
-        <v>-0.00177593741763038</v>
+        <v>-0.001775937417630269</v>
       </c>
       <c r="N17" t="n">
         <v>-0.1115079251282154</v>
       </c>
       <c r="O17" t="n">
-        <v>-0.1239615861782468</v>
+        <v>-0.123961586178325</v>
       </c>
       <c r="P17" t="n">
-        <v>-2.585323163895037e-05</v>
+        <v>3.298918492544711e-05</v>
       </c>
     </row>
     <row r="18">
@@ -5831,7 +5831,7 @@
         <v>-0.276015000000001</v>
       </c>
       <c r="K18" t="n">
-        <v>-1.011492910607537e-05</v>
+        <v>-0.000483046520226238</v>
       </c>
       <c r="L18" t="n">
         <v>-0.003852166103913368</v>
@@ -5843,10 +5843,10 @@
         <v>-1.352777204972206</v>
       </c>
       <c r="O18" t="n">
-        <v>-1.172265986974786</v>
+        <v>-1.172265986974587</v>
       </c>
       <c r="P18" t="n">
-        <v>-1.00096325506005e-05</v>
+        <v>-0.0004830196744374238</v>
       </c>
     </row>
     <row r="19">
@@ -5883,7 +5883,7 @@
         <v>0.08583400000000552</v>
       </c>
       <c r="K19" t="n">
-        <v>-2.850395524445215e-05</v>
+        <v>-0.001044512090183192</v>
       </c>
       <c r="L19" t="n">
         <v>-0.009216926301165107</v>
@@ -5895,10 +5895,10 @@
         <v>-1.010188250301532</v>
       </c>
       <c r="O19" t="n">
-        <v>-0.959965241321548</v>
+        <v>-0.9599652413214343</v>
       </c>
       <c r="P19" t="n">
-        <v>-2.852276102061069e-05</v>
+        <v>-0.001044515645653554</v>
       </c>
     </row>
     <row r="20">
@@ -5935,22 +5935,22 @@
         <v>0.08519400000000132</v>
       </c>
       <c r="K20" t="n">
-        <v>-8.644439631444456e-06</v>
+        <v>-0.0001451572925351696</v>
       </c>
       <c r="L20" t="n">
         <v>-0.001174589465786524</v>
       </c>
       <c r="M20" t="n">
-        <v>-0.001059914511747029</v>
+        <v>-0.001059914511746807</v>
       </c>
       <c r="N20" t="n">
         <v>-0.07807828422205176</v>
       </c>
       <c r="O20" t="n">
-        <v>-0.08749561520064475</v>
+        <v>-0.0874956152007158</v>
       </c>
       <c r="P20" t="n">
-        <v>-8.246467115724521e-06</v>
+        <v>-0.0001450900833566138</v>
       </c>
     </row>
     <row r="21">
@@ -5987,7 +5987,7 @@
         <v>-0.7220079999999882</v>
       </c>
       <c r="K21" t="n">
-        <v>2.543103361341004e-06</v>
+        <v>3.876247168943525e-05</v>
       </c>
       <c r="L21" t="n">
         <v>-0.0001044368175164845</v>
@@ -5999,10 +5999,10 @@
         <v>-0.01300037364615747</v>
       </c>
       <c r="O21" t="n">
-        <v>-0.02632134747382509</v>
+        <v>-0.02632134747381087</v>
       </c>
       <c r="P21" t="n">
-        <v>2.898076678192751e-06</v>
+        <v>3.88025137517678e-05</v>
       </c>
     </row>
   </sheetData>
@@ -6187,7 +6187,7 @@
         <v>15.10169090120603</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.6186184032803365</v>
+        <v>-0.6186184032803366</v>
       </c>
       <c r="G2" t="n">
         <v>-0.902413792110287</v>
@@ -6243,7 +6243,7 @@
         <v>14.83187700670705</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.578270630332773</v>
+        <v>-0.5782706303327729</v>
       </c>
       <c r="G4" t="n">
         <v>-0.881628071292377</v>
@@ -6262,7 +6262,7 @@
         <v>5</v>
       </c>
       <c r="C5" t="n">
-        <v>3.256166018976243</v>
+        <v>3.256166018976244</v>
       </c>
       <c r="D5" t="n">
         <v>0.114771913641154</v>
@@ -6271,7 +6271,7 @@
         <v>7.565728235600844</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.1662350155305652</v>
+        <v>-0.1662350155305651</v>
       </c>
       <c r="G5" t="n">
         <v>-0.3248702821473083</v>
@@ -6290,22 +6290,22 @@
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>5.37109742217857</v>
+        <v>5.042590775915152</v>
       </c>
       <c r="D6" t="n">
-        <v>3.222272097232781</v>
+        <v>3.69604512444528</v>
       </c>
       <c r="E6" t="n">
-        <v>7.810305482788937</v>
+        <v>6.707913892247852</v>
       </c>
       <c r="F6" t="n">
-        <v>-5.027688225643041e-05</v>
+        <v>-0.0005140640925927607</v>
       </c>
       <c r="G6" t="n">
-        <v>-9.570958725147511e-05</v>
+        <v>-0.0006447576064173021</v>
       </c>
       <c r="H6" t="n">
-        <v>-1.907484293848989e-05</v>
+        <v>-0.0003764584430727145</v>
       </c>
     </row>
     <row r="7">
@@ -6346,22 +6346,22 @@
         <v>5</v>
       </c>
       <c r="C8" t="n">
-        <v>16.16607757942608</v>
+        <v>16.16607757942607</v>
       </c>
       <c r="D8" t="n">
-        <v>12.53249578643494</v>
+        <v>12.53249578643512</v>
       </c>
       <c r="E8" t="n">
-        <v>20.52844511731935</v>
+        <v>20.52844511731882</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.00415934068147054</v>
+        <v>-0.004159340681470542</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.007181607599020947</v>
+        <v>-0.007181607599020966</v>
       </c>
       <c r="H8" t="n">
-        <v>-0.002489664583250229</v>
+        <v>-0.002489664583250328</v>
       </c>
     </row>
     <row r="9">
@@ -6383,7 +6383,7 @@
         <v>15.37869562744516</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.5759191037454497</v>
+        <v>-0.5759191037454496</v>
       </c>
       <c r="G9" t="n">
         <v>-0.8469594665367928</v>
@@ -6402,22 +6402,22 @@
         <v>5</v>
       </c>
       <c r="C10" t="n">
-        <v>11.59486358502314</v>
+        <v>11.5948635850229</v>
       </c>
       <c r="D10" t="n">
-        <v>9.518747089939495</v>
+        <v>9.518747089940138</v>
       </c>
       <c r="E10" t="n">
-        <v>14.78593506351105</v>
+        <v>14.7859350635092</v>
       </c>
       <c r="F10" t="n">
         <v>-0.5694103445000935</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.845343709229918</v>
+        <v>-0.8453437092299368</v>
       </c>
       <c r="H10" t="n">
-        <v>-0.3743202841450572</v>
+        <v>-0.374320284145072</v>
       </c>
     </row>
     <row r="11">
@@ -6430,22 +6430,22 @@
         <v>5</v>
       </c>
       <c r="C11" t="n">
-        <v>5.365538398127909</v>
+        <v>5.042616008145933</v>
       </c>
       <c r="D11" t="n">
-        <v>3.221943170765629</v>
+        <v>3.696054410679395</v>
       </c>
       <c r="E11" t="n">
-        <v>7.821265077839268</v>
+        <v>6.708015764553266</v>
       </c>
       <c r="F11" t="n">
-        <v>-5.026448906507506e-05</v>
+        <v>-0.0005140715790043322</v>
       </c>
       <c r="G11" t="n">
-        <v>-9.557335451100943e-05</v>
+        <v>-0.0006447461264400202</v>
       </c>
       <c r="H11" t="n">
-        <v>-1.894793491599015e-05</v>
+        <v>-0.0003764525371620529</v>
       </c>
     </row>
   </sheetData>

</xml_diff>